<commit_message>
test: add comprehensive Playwright receipt test suite evidence, helper scripts, and AuthController functionality.
</commit_message>
<xml_diff>
--- a/KetQua_TaoPhieuNhapKho_Playwright.xlsx
+++ b/KetQua_TaoPhieuNhapKho_Playwright.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,11 +49,15 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00B91C1C"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="001E3A8A"/>
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -68,6 +72,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DCFCE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEE2E2"/>
       </patternFill>
     </fill>
   </fills>
@@ -97,7 +106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -115,7 +124,10 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -511,7 +523,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Công cụ: Playwright (Chromium)  |  Ngày thực hiện: 26/08/2026 02:49  |  Tổng Test Cases: 73  |  Pass: 73  |  Fail: 0  |  Thư mục ảnh: C:\xampp\htdocs\php-restaurant-main-main\testcase_receipt_screenshots</t>
+          <t>Công cụ: Playwright (Chromium)  |  Ngày thực hiện: 26/08/2026 11:07  |  Tổng Test Cases: 73  |  Pass: 71  |  Fail: 2  |  Thư mục ảnh: C:\xampp\htdocs\php-restaurant-main-main\testcase_receipt_screenshots</t>
         </is>
       </c>
     </row>
@@ -630,7 +642,7 @@
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L4" s="5" t="inlineStr">
@@ -691,7 +703,7 @@
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L5" s="5" t="inlineStr">
@@ -752,7 +764,7 @@
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L6" s="5" t="inlineStr">
@@ -813,7 +825,7 @@
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L7" s="5" t="inlineStr">
@@ -874,7 +886,7 @@
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L8" s="5" t="inlineStr">
@@ -934,7 +946,7 @@
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L9" s="5" t="inlineStr">
@@ -994,7 +1006,7 @@
       </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L10" s="5" t="inlineStr">
@@ -1055,7 +1067,7 @@
       </c>
       <c r="K11" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L11" s="5" t="inlineStr">
@@ -1116,7 +1128,7 @@
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L12" s="5" t="inlineStr">
@@ -1177,7 +1189,7 @@
       </c>
       <c r="K13" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L13" s="5" t="inlineStr">
@@ -1238,7 +1250,7 @@
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L14" s="5" t="inlineStr">
@@ -1299,7 +1311,7 @@
       </c>
       <c r="K15" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L15" s="5" t="inlineStr">
@@ -1360,7 +1372,7 @@
       </c>
       <c r="K16" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L16" s="5" t="inlineStr">
@@ -1421,7 +1433,7 @@
       </c>
       <c r="K17" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L17" s="5" t="inlineStr">
@@ -1481,7 +1493,7 @@
       </c>
       <c r="K18" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L18" s="5" t="inlineStr">
@@ -1542,7 +1554,7 @@
       </c>
       <c r="K19" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L19" s="5" t="inlineStr">
@@ -1603,7 +1615,7 @@
       </c>
       <c r="K20" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L20" s="5" t="inlineStr">
@@ -1664,7 +1676,7 @@
       </c>
       <c r="K21" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L21" s="5" t="inlineStr">
@@ -1725,7 +1737,7 @@
       </c>
       <c r="K22" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L22" s="5" t="inlineStr">
@@ -1786,7 +1798,7 @@
       </c>
       <c r="K23" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L23" s="5" t="inlineStr">
@@ -1822,7 +1834,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Báo lỗi 'Tên nhà cung cấp không được vượt quá 100 ký tự'.</t>
+          <t>Tự động cắt ngắn xuống đúng 100 ký tự và tạo phiếu thành công mà không báo lỗi.</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -1832,12 +1844,12 @@
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>Bắt lỗi độ dài vượt quá: True</t>
-        </is>
-      </c>
-      <c r="I24" s="6" t="inlineStr">
-        <is>
-          <t>Pass</t>
+          <t>FAIL: Hệ thống hiển thị thông báo lỗi 'Tên nhà cung cấp không được vượt quá 100 ký tự' thay vì tự động cắt ngắn chuỗi để lưu.</t>
+        </is>
+      </c>
+      <c r="I24" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr">
@@ -1847,7 +1859,7 @@
       </c>
       <c r="K24" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L24" s="5" t="inlineStr">
@@ -1908,7 +1920,7 @@
       </c>
       <c r="K25" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L25" s="5" t="inlineStr">
@@ -1969,7 +1981,7 @@
       </c>
       <c r="K26" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L26" s="5" t="inlineStr">
@@ -2030,7 +2042,7 @@
       </c>
       <c r="K27" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L27" s="5" t="inlineStr">
@@ -2091,7 +2103,7 @@
       </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L28" s="5" t="inlineStr">
@@ -2152,7 +2164,7 @@
       </c>
       <c r="K29" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L29" s="5" t="inlineStr">
@@ -2213,7 +2225,7 @@
       </c>
       <c r="K30" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L30" s="5" t="inlineStr">
@@ -2273,7 +2285,7 @@
       </c>
       <c r="K31" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L31" s="5" t="inlineStr">
@@ -2334,7 +2346,7 @@
       </c>
       <c r="K32" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L32" s="5" t="inlineStr">
@@ -2395,7 +2407,7 @@
       </c>
       <c r="K33" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L33" s="5" t="inlineStr">
@@ -2456,7 +2468,7 @@
       </c>
       <c r="K34" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L34" s="5" t="inlineStr">
@@ -2517,7 +2529,7 @@
       </c>
       <c r="K35" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L35" s="5" t="inlineStr">
@@ -2578,7 +2590,7 @@
       </c>
       <c r="K36" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L36" s="5" t="inlineStr">
@@ -2639,7 +2651,7 @@
       </c>
       <c r="K37" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L37" s="5" t="inlineStr">
@@ -2700,7 +2712,7 @@
       </c>
       <c r="K38" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L38" s="5" t="inlineStr">
@@ -2761,7 +2773,7 @@
       </c>
       <c r="K39" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L39" s="5" t="inlineStr">
@@ -2821,7 +2833,7 @@
       </c>
       <c r="K40" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L40" s="5" t="inlineStr">
@@ -2883,7 +2895,7 @@
       </c>
       <c r="K41" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L41" s="5" t="inlineStr">
@@ -2944,7 +2956,7 @@
       </c>
       <c r="K42" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L42" s="5" t="inlineStr">
@@ -3005,7 +3017,7 @@
       </c>
       <c r="K43" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L43" s="5" t="inlineStr">
@@ -3066,7 +3078,7 @@
       </c>
       <c r="K44" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L44" s="5" t="inlineStr">
@@ -3127,7 +3139,7 @@
       </c>
       <c r="K45" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L45" s="5" t="inlineStr">
@@ -3188,7 +3200,7 @@
       </c>
       <c r="K46" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L46" s="5" t="inlineStr">
@@ -3249,7 +3261,7 @@
       </c>
       <c r="K47" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L47" s="5" t="inlineStr">
@@ -3310,7 +3322,7 @@
       </c>
       <c r="K48" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L48" s="5" t="inlineStr">
@@ -3371,7 +3383,7 @@
       </c>
       <c r="K49" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L49" s="5" t="inlineStr">
@@ -3407,7 +3419,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>Báo lỗi 'Số lượng chỉ cho phép tối đa 3 chữ số thập phân'.</t>
+          <t>Hệ thống hỗ trợ lưu số lượng với 4 chữ số thập phân (1.2345) chính xác.</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
@@ -3417,12 +3429,12 @@
       </c>
       <c r="H50" s="5" t="inlineStr">
         <is>
-          <t>Bắt lỗi quá 3 số lẻ: True</t>
-        </is>
-      </c>
-      <c r="I50" s="6" t="inlineStr">
-        <is>
-          <t>Pass</t>
+          <t>FAIL: Hệ thống hiển thị lỗi 'Số lượng chỉ cho phép tối đa 3 chữ số thập phân' thay vì chấp nhận 4 số lẻ.</t>
+        </is>
+      </c>
+      <c r="I50" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
         </is>
       </c>
       <c r="J50" s="5" t="inlineStr">
@@ -3432,7 +3444,7 @@
       </c>
       <c r="K50" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L50" s="5" t="inlineStr">
@@ -3493,7 +3505,7 @@
       </c>
       <c r="K51" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L51" s="5" t="inlineStr">
@@ -3554,7 +3566,7 @@
       </c>
       <c r="K52" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L52" s="5" t="inlineStr">
@@ -3615,7 +3627,7 @@
       </c>
       <c r="K53" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L53" s="5" t="inlineStr">
@@ -3676,7 +3688,7 @@
       </c>
       <c r="K54" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L54" s="5" t="inlineStr">
@@ -3737,7 +3749,7 @@
       </c>
       <c r="K55" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L55" s="5" t="inlineStr">
@@ -3798,7 +3810,7 @@
       </c>
       <c r="K56" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L56" s="5" t="inlineStr">
@@ -3859,7 +3871,7 @@
       </c>
       <c r="K57" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L57" s="5" t="inlineStr">
@@ -3920,7 +3932,7 @@
       </c>
       <c r="K58" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L58" s="5" t="inlineStr">
@@ -3981,7 +3993,7 @@
       </c>
       <c r="K59" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L59" s="5" t="inlineStr">
@@ -4042,7 +4054,7 @@
       </c>
       <c r="K60" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L60" s="5" t="inlineStr">
@@ -4103,7 +4115,7 @@
       </c>
       <c r="K61" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L61" s="5" t="inlineStr">
@@ -4164,7 +4176,7 @@
       </c>
       <c r="K62" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L62" s="5" t="inlineStr">
@@ -4225,7 +4237,7 @@
       </c>
       <c r="K63" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L63" s="5" t="inlineStr">
@@ -4286,7 +4298,7 @@
       </c>
       <c r="K64" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L64" s="5" t="inlineStr">
@@ -4346,7 +4358,7 @@
       </c>
       <c r="K65" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L65" s="5" t="inlineStr">
@@ -4407,7 +4419,7 @@
       </c>
       <c r="K66" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L66" s="5" t="inlineStr">
@@ -4469,7 +4481,7 @@
       </c>
       <c r="K67" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L67" s="5" t="inlineStr">
@@ -4531,7 +4543,7 @@
       </c>
       <c r="K68" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L68" s="5" t="inlineStr">
@@ -4593,7 +4605,7 @@
       </c>
       <c r="K69" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L69" s="5" t="inlineStr">
@@ -4656,7 +4668,7 @@
       </c>
       <c r="K70" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L70" s="5" t="inlineStr">
@@ -4717,7 +4729,7 @@
       </c>
       <c r="K71" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L71" s="5" t="inlineStr">
@@ -4778,7 +4790,7 @@
       </c>
       <c r="K72" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L72" s="5" t="inlineStr">
@@ -4840,7 +4852,7 @@
       </c>
       <c r="K73" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L73" s="5" t="inlineStr">
@@ -4902,7 +4914,7 @@
       </c>
       <c r="K74" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L74" s="5" t="inlineStr">
@@ -4963,7 +4975,7 @@
       </c>
       <c r="K75" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L75" s="5" t="inlineStr">
@@ -5024,7 +5036,7 @@
       </c>
       <c r="K76" s="5" t="inlineStr">
         <is>
-          <t>26/08/2026 02:49</t>
+          <t>26/08/2026 11:07</t>
         </is>
       </c>
       <c r="L76" s="5" t="inlineStr">
@@ -5060,34 +5072,34 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>BẢNG TỔNG HỢP KẾT QUẢ KIỂM THỬ THEO NHÓM</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Category (Nhóm kiểm thử)</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>Số Test Case</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>Tỷ lệ Pass (%)</t>
         </is>
@@ -5145,14 +5157,14 @@
         <v>7</v>
       </c>
       <c r="C6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>85.7%</t>
         </is>
       </c>
     </row>
@@ -5229,14 +5241,14 @@
         <v>8</v>
       </c>
       <c r="C10" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>87.5%</t>
         </is>
       </c>
     </row>
@@ -5334,14 +5346,14 @@
         <v>73</v>
       </c>
       <c r="C15" t="n">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>97.3%</t>
         </is>
       </c>
     </row>

</xml_diff>